<commit_message>
Added us core v8.0.0 requirements. In the processes, noted some necessary changes to the v7.0.0 and v6.1.0 requirements. Updated these, regenerated the csv file, and regenerated the coverage file.
</commit_message>
<xml_diff>
--- a/lib/us_core_test_kit/requirements/hl7.fhir.us.core_6.1.0_reqs.xlsx
+++ b/lib/us_core_test_kit/requirements/hl7.fhir.us.core_6.1.0_reqs.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/knaden/Documents/Inferno/source/us-core-test-kit/lib/us_core_test_kit/requirements/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/edeyoung/Documents/inferno/us-core-test-kit/lib/us_core_test_kit/requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B26E4571-9F78-E84A-88DC-63B5BFA7F593}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9938CB48-E2A5-3A4B-A7F0-7485136FD2D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1780" yWindow="760" windowWidth="27360" windowHeight="20180" firstSheet="1" activeTab="2" xr2:uid="{D251129A-65BB-5042-909C-749E11B8C0B0}"/>
+    <workbookView xWindow="1780" yWindow="760" windowWidth="27360" windowHeight="18880" firstSheet="1" activeTab="1" xr2:uid="{D251129A-65BB-5042-909C-749E11B8C0B0}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="9" r:id="rId1"/>
@@ -77,7 +77,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -99,7 +99,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3047" uniqueCount="1060">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3044" uniqueCount="1061">
   <si>
     <r>
       <rPr>
@@ -4085,43 +4085,16 @@
     <t>https://hl7.org/fhir/us/core/STU6.1/StructureDefinition-us-core-patient.html#mandatory-and-must-support-data-elements, https://hl7.org/fhir/us/core/STU6.1/StructureDefinition-us-core-race.html#profile-specific-implementation-guidance</t>
   </si>
   <si>
-    <t>[Organizations participating in the ONC Health IT certrification program,] must support at least one category code from OMB Race [category for the [US Core Race Extension] (https://hl7.org/fhir/us/core/STU7/StructureDefinition-us-core-race.html)]</t>
-  </si>
-  <si>
-    <t>For organizations participating in ONC certification, when using the US Core Race Extension</t>
-  </si>
-  <si>
     <t>Deprecating as this is not in US 6.1,</t>
   </si>
   <si>
     <t>https://hl7.org/fhir/us/core/STU6.1/StructureDefinition-us-core-patient.html#mandatory-and-must-support-data-elements, https://hl7.org/fhir/us/core/STU6.1/StructureDefinition-us-core-ethnicity.html#profile-specific-implementation-guidance</t>
   </si>
   <si>
-    <t>[Organizations participating in the ONC Health IT certrification program,] must support at least one category code from OMB … Ethnicity [category for the [US Core Ethnicity Extension] (https://hl7.org/fhir/us/core/STU7/StructureDefinition-us-core-ethnicity.html)]</t>
-  </si>
-  <si>
-    <t>For organizations participating in ONC certification, When using the US Core Ethnicity Extension</t>
-  </si>
-  <si>
-    <t>[Organizations participating in the ONC Health IT certrification program,] MAY include additional detailed codes from CDC Race … codes [when using the [US Core Race Extension] (https://hl7.org/fhir/us/core/STU7/StructureDefinition-us-core-race.html)]</t>
-  </si>
-  <si>
-    <t>For organizations participating in ONC certification, When using the US Core Race Extension</t>
-  </si>
-  <si>
-    <t>[Organizations participating in the ONC Health IT certrification program,] SHALL include a text description [of category codes when using the [US Core Ethnicity Extension] (https://hl7.org/fhir/us/core/STU7/StructureDefinition-us-core-ethnicity.html)]</t>
-  </si>
-  <si>
     <t>Unknown</t>
   </si>
   <si>
     <t>https://hl7.org/fhir/us/core/STU6.1/StructureDefinition-us-core-patient.html#mandatory-and-must-support-data-elements</t>
-  </si>
-  <si>
-    <t>[For Organizations participating in the ONC Health IT certrification program,] Although Patient.deceased[x] is marked as additional USCDI, certifying systems are not required to support both [boolean and dateTime data types], but SHALL support [at] least Patient.deceasedDateTime</t>
-  </si>
-  <si>
-    <t xml:space="preserve">For organizations participating in ONC certification, </t>
   </si>
   <si>
     <t>Previous name is represented by setting Patient.name.use to “old” or providing an end date in Patient.name.period or doing both</t>
@@ -4872,12 +4845,42 @@
   <si>
     <t>hl7.fhir.us.core_6.1.0</t>
   </si>
+  <si>
+    <t>Marked DEPRECATED because this is an example.</t>
+  </si>
+  <si>
+    <t>Duplicate of 254</t>
+  </si>
+  <si>
+    <t>Duplicate of requirement 260</t>
+  </si>
+  <si>
+    <t>The Complex [Extension] for Race ... allow[s] for one or more codes of which must support at least one category code from OMB Race [category for the [US Core Race Extension] (https://hl7.org/fhir/us/core/STU7/StructureDefinition-us-core-race.html)]</t>
+  </si>
+  <si>
+    <t>The Complex [Extension] for ... Ethnicity allow[s] for one or more codes of which must support at least one category code from OMB … Ethnicity [category for the [US Core Ethnicity Extension] (https://hl7.org/fhir/us/core/STU7/StructureDefinition-us-core-ethnicity.html)]</t>
+  </si>
+  <si>
+    <t>The Complex [Extension] for Race ... allow[s] for one or more codes of which MAY include additional detailed codes from CDC Race … codes [when using the [US Core Race Extension] (https://hl7.org/fhir/us/core/STU7/StructureDefinition-us-core-race.html)]</t>
+  </si>
+  <si>
+    <t>The Complex [Extension] for Race ... allow[s] for one or more codes of which SHALL include a text description [of category codes when using the [US Core Race Extension] (https://hl7.org/fhir/us/core/STU7/StructureDefinition-us-core-race.html)]</t>
+  </si>
+  <si>
+    <t>The Complex [Extension] for ... Ethnicity allow[s] for one or more codes of which MAY include additional detailed codes from CDC Race … codes [when using the [US Core Race Extension] (https://hl7.org/fhir/us/core/STU7/StructureDefinition-us-core-race.html)]</t>
+  </si>
+  <si>
+    <t>The Complex [Extension] for ... Ethnicity allow[s] for one or more codes of which SHALL include a text description [of category codes when using the [US Core Ethnicity Extension] (https://hl7.org/fhir/us/core/STU7/StructureDefinition-us-core-ethnicity.html)]</t>
+  </si>
+  <si>
+    <t>Although Patient.deceased[x] is marked as additional USCDI, certifying systems are not required to support both [boolean and dateTime data types], but SHALL support [at] least Patient.deceasedDateTime</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="24" x14ac:knownFonts="1">
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -5041,8 +5044,15 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -5103,8 +5113,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFDA"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="22">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -5359,12 +5375,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0CECE"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0CECE"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0CECE"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD0CECE"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5523,6 +5554,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -9892,8 +9926,8 @@
       <c r="A94" s="7">
         <v>87</v>
       </c>
-      <c r="B94" s="7" t="s">
-        <v>195</v>
+      <c r="B94" s="23" t="s">
+        <v>209</v>
       </c>
       <c r="C94" s="8" t="s">
         <v>207</v>
@@ -9913,7 +9947,7 @@
       </c>
       <c r="N94" s="9" t="str" cm="1">
         <f t="array" ref="N94">SECTION_NAME(B94)</f>
-        <v>additional-uscdi-requirements</v>
+        <v>defined-pattern-elements</v>
       </c>
       <c r="O94" s="10" t="str">
         <f t="shared" si="4"/>
@@ -9939,7 +9973,7 @@
         <v>210</v>
       </c>
       <c r="D95" s="7" t="s">
-        <v>32</v>
+        <v>87</v>
       </c>
       <c r="E95" s="7" t="s">
         <v>33</v>
@@ -9966,6 +10000,9 @@
         <f t="shared" si="3"/>
         <v>Server</v>
       </c>
+      <c r="T95" s="13" t="s">
+        <v>1051</v>
+      </c>
       <c r="U95" s="63"/>
     </row>
     <row r="96" spans="1:21" ht="187" x14ac:dyDescent="0.2">
@@ -9979,7 +10016,7 @@
         <v>212</v>
       </c>
       <c r="D96" s="7" t="s">
-        <v>32</v>
+        <v>87</v>
       </c>
       <c r="E96" s="7" t="s">
         <v>79</v>
@@ -10005,6 +10042,9 @@
       <c r="P96" s="10" t="str">
         <f t="shared" si="3"/>
         <v>Client</v>
+      </c>
+      <c r="T96" s="13" t="s">
+        <v>1051</v>
       </c>
       <c r="U96" s="63"/>
     </row>
@@ -16751,7 +16791,7 @@
         <v>513</v>
       </c>
       <c r="D263" s="7" t="s">
-        <v>32</v>
+        <v>87</v>
       </c>
       <c r="E263" s="7" t="s">
         <v>33</v>
@@ -16778,6 +16818,9 @@
       <c r="Q263" s="10" t="s">
         <v>514</v>
       </c>
+      <c r="T263" s="56" t="s">
+        <v>1052</v>
+      </c>
       <c r="U263" s="63"/>
     </row>
     <row r="264" spans="1:21" ht="306" x14ac:dyDescent="0.2">
@@ -16954,7 +16997,7 @@
         <v>33</v>
       </c>
       <c r="G268" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M268" s="9" t="str" cm="1">
         <f t="array" ref="M268">PAGE_NAME(B268)</f>
@@ -16988,7 +17031,7 @@
         <v>521</v>
       </c>
       <c r="D269" s="7" t="s">
-        <v>32</v>
+        <v>87</v>
       </c>
       <c r="E269" s="7" t="s">
         <v>33</v>
@@ -17015,6 +17058,9 @@
       <c r="Q269" s="10" t="s">
         <v>522</v>
       </c>
+      <c r="T269" s="71" t="s">
+        <v>1053</v>
+      </c>
       <c r="U269" s="63"/>
     </row>
     <row r="270" spans="1:21" ht="238" x14ac:dyDescent="0.2">
@@ -24613,7 +24659,7 @@
         <v>867</v>
       </c>
       <c r="C467" s="8" t="s">
-        <v>868</v>
+        <v>1054</v>
       </c>
       <c r="D467" s="7" t="s">
         <v>87</v>
@@ -24623,9 +24669,6 @@
       </c>
       <c r="G467" s="7" t="b">
         <v>1</v>
-      </c>
-      <c r="H467" s="13" t="s">
-        <v>869</v>
       </c>
       <c r="M467" s="9" t="str" cm="1">
         <f t="array" ref="M467">PAGE_NAME(B467)</f>
@@ -24644,7 +24687,7 @@
         <v/>
       </c>
       <c r="U467" s="13" t="s">
-        <v>870</v>
+        <v>868</v>
       </c>
     </row>
     <row r="468" spans="1:21" ht="102" x14ac:dyDescent="0.2">
@@ -24652,10 +24695,10 @@
         <v>460</v>
       </c>
       <c r="B468" s="23" t="s">
-        <v>871</v>
+        <v>869</v>
       </c>
       <c r="C468" s="8" t="s">
-        <v>872</v>
+        <v>1055</v>
       </c>
       <c r="D468" s="7" t="s">
         <v>87</v>
@@ -24665,9 +24708,6 @@
       </c>
       <c r="G468" s="7" t="b">
         <v>1</v>
-      </c>
-      <c r="H468" s="13" t="s">
-        <v>873</v>
       </c>
       <c r="M468" s="9" t="str" cm="1">
         <f t="array" ref="M468">PAGE_NAME(B468)</f>
@@ -24686,7 +24726,7 @@
         <v/>
       </c>
       <c r="U468" s="13" t="s">
-        <v>870</v>
+        <v>868</v>
       </c>
     </row>
     <row r="469" spans="1:21" ht="102" x14ac:dyDescent="0.2">
@@ -24697,7 +24737,7 @@
         <v>867</v>
       </c>
       <c r="C469" s="8" t="s">
-        <v>874</v>
+        <v>1056</v>
       </c>
       <c r="D469" s="7" t="s">
         <v>87</v>
@@ -24707,9 +24747,6 @@
       </c>
       <c r="G469" s="7" t="b">
         <v>1</v>
-      </c>
-      <c r="H469" s="13" t="s">
-        <v>875</v>
       </c>
       <c r="M469" s="9" t="str" cm="1">
         <f t="array" ref="M469">PAGE_NAME(B469)</f>
@@ -24728,7 +24765,7 @@
         <v/>
       </c>
       <c r="U469" s="13" t="s">
-        <v>870</v>
+        <v>868</v>
       </c>
     </row>
     <row r="470" spans="1:21" ht="102" x14ac:dyDescent="0.2">
@@ -24736,10 +24773,10 @@
         <v>462</v>
       </c>
       <c r="B470" s="23" t="s">
-        <v>871</v>
+        <v>869</v>
       </c>
       <c r="C470" s="8" t="s">
-        <v>876</v>
+        <v>1057</v>
       </c>
       <c r="D470" s="7" t="s">
         <v>87</v>
@@ -24749,9 +24786,6 @@
       </c>
       <c r="G470" s="7" t="b">
         <v>1</v>
-      </c>
-      <c r="H470" s="13" t="s">
-        <v>873</v>
       </c>
       <c r="M470" s="9" t="str" cm="1">
         <f t="array" ref="M470">PAGE_NAME(B470)</f>
@@ -24770,7 +24804,7 @@
         <v/>
       </c>
       <c r="U470" s="13" t="s">
-        <v>870</v>
+        <v>868</v>
       </c>
     </row>
     <row r="471" spans="1:21" ht="102" x14ac:dyDescent="0.2">
@@ -24781,7 +24815,7 @@
         <v>867</v>
       </c>
       <c r="C471" s="8" t="s">
-        <v>874</v>
+        <v>1058</v>
       </c>
       <c r="D471" s="7" t="s">
         <v>87</v>
@@ -24791,9 +24825,6 @@
       </c>
       <c r="G471" s="7" t="b">
         <v>1</v>
-      </c>
-      <c r="H471" s="13" t="s">
-        <v>875</v>
       </c>
       <c r="M471" s="9" t="str" cm="1">
         <f t="array" ref="M471">PAGE_NAME(B471)</f>
@@ -24812,7 +24843,7 @@
         <v/>
       </c>
       <c r="U471" s="13" t="s">
-        <v>870</v>
+        <v>868</v>
       </c>
     </row>
     <row r="472" spans="1:21" ht="102" x14ac:dyDescent="0.2">
@@ -24820,10 +24851,10 @@
         <v>464</v>
       </c>
       <c r="B472" s="23" t="s">
-        <v>871</v>
+        <v>869</v>
       </c>
       <c r="C472" s="8" t="s">
-        <v>876</v>
+        <v>1059</v>
       </c>
       <c r="D472" s="7" t="s">
         <v>87</v>
@@ -24833,9 +24864,6 @@
       </c>
       <c r="G472" s="7" t="b">
         <v>1</v>
-      </c>
-      <c r="H472" s="13" t="s">
-        <v>873</v>
       </c>
       <c r="M472" s="9" t="str" cm="1">
         <f t="array" ref="M472">PAGE_NAME(B472)</f>
@@ -24854,27 +24882,24 @@
         <v/>
       </c>
       <c r="U472" s="13" t="s">
-        <v>870</v>
-      </c>
-    </row>
-    <row r="473" spans="1:21" ht="119" x14ac:dyDescent="0.2">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="473" spans="1:21" ht="85" x14ac:dyDescent="0.2">
       <c r="A473" s="7">
         <v>465</v>
       </c>
       <c r="B473" s="23" t="s">
-        <v>878</v>
+        <v>871</v>
       </c>
       <c r="C473" s="8" t="s">
-        <v>879</v>
+        <v>1060</v>
       </c>
       <c r="D473" s="7" t="s">
         <v>87</v>
       </c>
       <c r="E473" s="7" t="s">
         <v>33</v>
-      </c>
-      <c r="H473" s="13" t="s">
-        <v>880</v>
       </c>
       <c r="M473" s="9" t="str" cm="1">
         <f t="array" ref="M473">PAGE_NAME(B473)</f>
@@ -24893,7 +24918,7 @@
         <v/>
       </c>
       <c r="U473" s="13" t="s">
-        <v>870</v>
+        <v>868</v>
       </c>
     </row>
     <row r="474" spans="1:21" ht="85" x14ac:dyDescent="0.2">
@@ -24901,10 +24926,10 @@
         <v>466</v>
       </c>
       <c r="B474" s="23" t="s">
-        <v>878</v>
+        <v>871</v>
       </c>
       <c r="C474" s="8" t="s">
-        <v>881</v>
+        <v>872</v>
       </c>
       <c r="D474" s="7" t="s">
         <v>37</v>
@@ -24916,7 +24941,7 @@
         <v>1</v>
       </c>
       <c r="H474" s="13" t="s">
-        <v>882</v>
+        <v>873</v>
       </c>
       <c r="O474" s="10" t="str">
         <f t="shared" si="23"/>
@@ -24932,10 +24957,10 @@
         <v>467</v>
       </c>
       <c r="B475" s="23" t="s">
-        <v>878</v>
+        <v>871</v>
       </c>
       <c r="C475" s="8" t="s">
-        <v>883</v>
+        <v>874</v>
       </c>
       <c r="D475" s="7" t="s">
         <v>37</v>
@@ -24947,7 +24972,7 @@
         <v>1</v>
       </c>
       <c r="H475" s="13" t="s">
-        <v>884</v>
+        <v>875</v>
       </c>
       <c r="M475" s="9" t="str" cm="1">
         <f t="array" ref="M475">PAGE_NAME(B475)</f>
@@ -24971,10 +24996,10 @@
         <v>468</v>
       </c>
       <c r="B476" s="23" t="s">
-        <v>878</v>
+        <v>871</v>
       </c>
       <c r="C476" s="8" t="s">
-        <v>885</v>
+        <v>876</v>
       </c>
       <c r="D476" s="7" t="s">
         <v>41</v>
@@ -25007,10 +25032,10 @@
         <v>469</v>
       </c>
       <c r="B477" s="23" t="s">
-        <v>878</v>
+        <v>871</v>
       </c>
       <c r="C477" s="8" t="s">
-        <v>886</v>
+        <v>877</v>
       </c>
       <c r="D477" s="7" t="s">
         <v>87</v>
@@ -25046,10 +25071,10 @@
         <v>470</v>
       </c>
       <c r="B478" s="23" t="s">
+        <v>871</v>
+      </c>
+      <c r="C478" s="8" t="s">
         <v>878</v>
-      </c>
-      <c r="C478" s="8" t="s">
-        <v>887</v>
       </c>
       <c r="D478" s="7" t="s">
         <v>87</v>
@@ -25085,10 +25110,10 @@
         <v>471</v>
       </c>
       <c r="B479" s="23" t="s">
-        <v>878</v>
+        <v>871</v>
       </c>
       <c r="C479" s="8" t="s">
-        <v>888</v>
+        <v>879</v>
       </c>
       <c r="D479" s="7" t="s">
         <v>87</v>
@@ -25100,7 +25125,7 @@
         <v>1</v>
       </c>
       <c r="H479" s="13" t="s">
-        <v>889</v>
+        <v>880</v>
       </c>
       <c r="M479" s="9" t="str" cm="1">
         <f t="array" ref="M479">PAGE_NAME(B479)</f>
@@ -25127,10 +25152,10 @@
         <v>472</v>
       </c>
       <c r="B480" s="23" t="s">
-        <v>878</v>
+        <v>871</v>
       </c>
       <c r="C480" s="8" t="s">
-        <v>890</v>
+        <v>881</v>
       </c>
       <c r="D480" s="7" t="s">
         <v>112</v>
@@ -25163,10 +25188,10 @@
         <v>473</v>
       </c>
       <c r="B481" s="23" t="s">
-        <v>891</v>
+        <v>882</v>
       </c>
       <c r="C481" s="8" t="s">
-        <v>892</v>
+        <v>883</v>
       </c>
       <c r="D481" s="7" t="s">
         <v>32</v>
@@ -25178,7 +25203,7 @@
         <v>1</v>
       </c>
       <c r="H481" s="13" t="s">
-        <v>893</v>
+        <v>884</v>
       </c>
       <c r="M481" s="9" t="str" cm="1">
         <f t="array" ref="M481">PAGE_NAME(B481)</f>
@@ -25202,10 +25227,10 @@
         <v>474</v>
       </c>
       <c r="B482" s="23" t="s">
-        <v>891</v>
+        <v>882</v>
       </c>
       <c r="C482" s="8" t="s">
-        <v>894</v>
+        <v>885</v>
       </c>
       <c r="D482" s="7" t="s">
         <v>87</v>
@@ -25217,7 +25242,7 @@
         <v>1</v>
       </c>
       <c r="H482" s="13" t="s">
-        <v>895</v>
+        <v>886</v>
       </c>
       <c r="M482" s="9" t="str" cm="1">
         <f t="array" ref="M482">PAGE_NAME(B482)</f>
@@ -25236,7 +25261,7 @@
         <v>Server</v>
       </c>
       <c r="U482" s="13" t="s">
-        <v>870</v>
+        <v>868</v>
       </c>
     </row>
     <row r="483" spans="1:21" ht="68" x14ac:dyDescent="0.2">
@@ -25244,10 +25269,10 @@
         <v>475</v>
       </c>
       <c r="B483" s="23" t="s">
-        <v>891</v>
+        <v>882</v>
       </c>
       <c r="C483" s="8" t="s">
-        <v>896</v>
+        <v>887</v>
       </c>
       <c r="D483" s="7" t="s">
         <v>87</v>
@@ -25259,7 +25284,7 @@
         <v>1</v>
       </c>
       <c r="H483" s="13" t="s">
-        <v>897</v>
+        <v>888</v>
       </c>
       <c r="M483" s="9" t="str" cm="1">
         <f t="array" ref="M483">PAGE_NAME(B483)</f>
@@ -25278,7 +25303,7 @@
         <v>Server</v>
       </c>
       <c r="U483" s="13" t="s">
-        <v>870</v>
+        <v>868</v>
       </c>
     </row>
     <row r="484" spans="1:21" ht="51" x14ac:dyDescent="0.2">
@@ -25286,10 +25311,10 @@
         <v>476</v>
       </c>
       <c r="B484" s="23" t="s">
-        <v>891</v>
+        <v>882</v>
       </c>
       <c r="C484" s="8" t="s">
-        <v>898</v>
+        <v>889</v>
       </c>
       <c r="D484" s="7" t="s">
         <v>87</v>
@@ -25314,7 +25339,7 @@
         <v>Client</v>
       </c>
       <c r="U484" s="13" t="s">
-        <v>899</v>
+        <v>890</v>
       </c>
     </row>
     <row r="485" spans="1:21" ht="51" x14ac:dyDescent="0.2">
@@ -25322,10 +25347,10 @@
         <v>477</v>
       </c>
       <c r="B485" s="23" t="s">
+        <v>882</v>
+      </c>
+      <c r="C485" s="8" t="s">
         <v>891</v>
-      </c>
-      <c r="C485" s="8" t="s">
-        <v>900</v>
       </c>
       <c r="D485" s="7" t="s">
         <v>37</v>
@@ -25358,10 +25383,10 @@
         <v>478</v>
       </c>
       <c r="B486" s="23" t="s">
-        <v>891</v>
+        <v>882</v>
       </c>
       <c r="C486" s="8" t="s">
-        <v>901</v>
+        <v>892</v>
       </c>
       <c r="D486" s="7" t="s">
         <v>87</v>
@@ -25397,10 +25422,10 @@
         <v>479</v>
       </c>
       <c r="B487" s="23" t="s">
-        <v>902</v>
+        <v>893</v>
       </c>
       <c r="C487" s="8" t="s">
-        <v>903</v>
+        <v>894</v>
       </c>
       <c r="D487" s="7" t="s">
         <v>41</v>
@@ -25433,10 +25458,10 @@
         <v>480</v>
       </c>
       <c r="B488" s="23" t="s">
-        <v>902</v>
+        <v>893</v>
       </c>
       <c r="C488" s="8" t="s">
-        <v>904</v>
+        <v>895</v>
       </c>
       <c r="D488" s="7" t="s">
         <v>37</v>
@@ -25448,7 +25473,7 @@
         <v>1</v>
       </c>
       <c r="H488" s="13" t="s">
-        <v>905</v>
+        <v>896</v>
       </c>
       <c r="M488" s="9" t="str" cm="1">
         <f t="array" ref="M488">PAGE_NAME(B488)</f>
@@ -25472,10 +25497,10 @@
         <v>481</v>
       </c>
       <c r="B489" s="23" t="s">
-        <v>902</v>
+        <v>893</v>
       </c>
       <c r="C489" s="8" t="s">
-        <v>906</v>
+        <v>897</v>
       </c>
       <c r="D489" s="7" t="s">
         <v>37</v>
@@ -25508,10 +25533,10 @@
         <v>482</v>
       </c>
       <c r="B490" s="23" t="s">
-        <v>902</v>
+        <v>893</v>
       </c>
       <c r="C490" s="8" t="s">
-        <v>907</v>
+        <v>898</v>
       </c>
       <c r="D490" s="7" t="s">
         <v>87</v>
@@ -25523,7 +25548,7 @@
         <v>1</v>
       </c>
       <c r="H490" s="13" t="s">
-        <v>908</v>
+        <v>899</v>
       </c>
       <c r="M490" s="9" t="str" cm="1">
         <f t="array" ref="M490">PAGE_NAME(B490)</f>
@@ -25542,7 +25567,7 @@
         <v>Server</v>
       </c>
       <c r="U490" s="13" t="s">
-        <v>899</v>
+        <v>890</v>
       </c>
     </row>
     <row r="491" spans="1:21" ht="85" x14ac:dyDescent="0.2">
@@ -25550,10 +25575,10 @@
         <v>483</v>
       </c>
       <c r="B491" s="23" t="s">
-        <v>902</v>
+        <v>893</v>
       </c>
       <c r="C491" s="8" t="s">
-        <v>909</v>
+        <v>900</v>
       </c>
       <c r="D491" s="7" t="s">
         <v>87</v>
@@ -25565,7 +25590,7 @@
         <v>1</v>
       </c>
       <c r="H491" s="13" t="s">
-        <v>908</v>
+        <v>899</v>
       </c>
       <c r="M491" s="9" t="str" cm="1">
         <f t="array" ref="M491">PAGE_NAME(B491)</f>
@@ -25584,7 +25609,7 @@
         <v>Client</v>
       </c>
       <c r="U491" s="13" t="s">
-        <v>899</v>
+        <v>890</v>
       </c>
     </row>
     <row r="492" spans="1:21" ht="119" x14ac:dyDescent="0.2">
@@ -25592,10 +25617,10 @@
         <v>484</v>
       </c>
       <c r="B492" s="23" t="s">
-        <v>902</v>
+        <v>893</v>
       </c>
       <c r="C492" s="8" t="s">
-        <v>910</v>
+        <v>901</v>
       </c>
       <c r="D492" s="7" t="s">
         <v>87</v>
@@ -25607,7 +25632,7 @@
         <v>1</v>
       </c>
       <c r="H492" s="13" t="s">
-        <v>911</v>
+        <v>902</v>
       </c>
       <c r="M492" s="9" t="str" cm="1">
         <f t="array" ref="M492">PAGE_NAME(B492)</f>
@@ -25626,7 +25651,7 @@
         <v>Server</v>
       </c>
       <c r="U492" s="13" t="s">
-        <v>899</v>
+        <v>890</v>
       </c>
     </row>
     <row r="493" spans="1:21" ht="85" x14ac:dyDescent="0.2">
@@ -25634,10 +25659,10 @@
         <v>485</v>
       </c>
       <c r="B493" s="23" t="s">
-        <v>902</v>
+        <v>893</v>
       </c>
       <c r="C493" s="8" t="s">
-        <v>912</v>
+        <v>903</v>
       </c>
       <c r="D493" s="7" t="s">
         <v>87</v>
@@ -25649,7 +25674,7 @@
         <v>1</v>
       </c>
       <c r="H493" s="13" t="s">
-        <v>908</v>
+        <v>899</v>
       </c>
       <c r="M493" s="9" t="str" cm="1">
         <f t="array" ref="M493">PAGE_NAME(B493)</f>
@@ -25668,7 +25693,7 @@
         <v>Client</v>
       </c>
       <c r="U493" s="13" t="s">
-        <v>899</v>
+        <v>890</v>
       </c>
     </row>
     <row r="494" spans="1:21" ht="85" x14ac:dyDescent="0.2">
@@ -25676,10 +25701,10 @@
         <v>486</v>
       </c>
       <c r="B494" s="23" t="s">
-        <v>902</v>
+        <v>893</v>
       </c>
       <c r="C494" s="8" t="s">
-        <v>913</v>
+        <v>904</v>
       </c>
       <c r="D494" s="7" t="s">
         <v>87</v>
@@ -25691,7 +25716,7 @@
         <v>1</v>
       </c>
       <c r="H494" s="13" t="s">
-        <v>914</v>
+        <v>905</v>
       </c>
       <c r="M494" s="9" t="str" cm="1">
         <f t="array" ref="M494">PAGE_NAME(B494)</f>
@@ -25710,7 +25735,7 @@
         <v>Server</v>
       </c>
       <c r="U494" s="13" t="s">
-        <v>899</v>
+        <v>890</v>
       </c>
     </row>
     <row r="495" spans="1:21" ht="85" x14ac:dyDescent="0.2">
@@ -25718,10 +25743,10 @@
         <v>487</v>
       </c>
       <c r="B495" s="23" t="s">
-        <v>902</v>
+        <v>893</v>
       </c>
       <c r="C495" s="8" t="s">
-        <v>915</v>
+        <v>906</v>
       </c>
       <c r="D495" s="7" t="s">
         <v>87</v>
@@ -25733,7 +25758,7 @@
         <v>1</v>
       </c>
       <c r="H495" s="13" t="s">
-        <v>914</v>
+        <v>905</v>
       </c>
       <c r="M495" s="9" t="str" cm="1">
         <f t="array" ref="M495">PAGE_NAME(B495)</f>
@@ -25752,7 +25777,7 @@
         <v>Client</v>
       </c>
       <c r="U495" s="13" t="s">
-        <v>899</v>
+        <v>890</v>
       </c>
     </row>
     <row r="496" spans="1:21" ht="119" x14ac:dyDescent="0.2">
@@ -25760,10 +25785,10 @@
         <v>488</v>
       </c>
       <c r="B496" s="23" t="s">
-        <v>902</v>
+        <v>893</v>
       </c>
       <c r="C496" s="8" t="s">
-        <v>916</v>
+        <v>907</v>
       </c>
       <c r="D496" s="7" t="s">
         <v>87</v>
@@ -25775,7 +25800,7 @@
         <v>1</v>
       </c>
       <c r="H496" s="13" t="s">
-        <v>914</v>
+        <v>905</v>
       </c>
       <c r="M496" s="9" t="str" cm="1">
         <f t="array" ref="M496">PAGE_NAME(B496)</f>
@@ -25794,7 +25819,7 @@
         <v/>
       </c>
       <c r="U496" s="13" t="s">
-        <v>899</v>
+        <v>890</v>
       </c>
     </row>
     <row r="497" spans="1:16" ht="51" x14ac:dyDescent="0.2">
@@ -25802,10 +25827,10 @@
         <v>489</v>
       </c>
       <c r="B497" s="23" t="s">
-        <v>917</v>
+        <v>908</v>
       </c>
       <c r="C497" s="8" t="s">
-        <v>918</v>
+        <v>909</v>
       </c>
       <c r="D497" s="7" t="s">
         <v>32</v>
@@ -25838,10 +25863,10 @@
         <v>490</v>
       </c>
       <c r="B498" s="23" t="s">
-        <v>917</v>
+        <v>908</v>
       </c>
       <c r="C498" s="8" t="s">
-        <v>919</v>
+        <v>910</v>
       </c>
       <c r="D498" s="7" t="s">
         <v>32</v>
@@ -25874,10 +25899,10 @@
         <v>491</v>
       </c>
       <c r="B499" s="23" t="s">
-        <v>917</v>
+        <v>908</v>
       </c>
       <c r="C499" s="8" t="s">
-        <v>920</v>
+        <v>911</v>
       </c>
       <c r="D499" s="7" t="s">
         <v>32</v>
@@ -25910,10 +25935,10 @@
         <v>492</v>
       </c>
       <c r="B500" s="23" t="s">
-        <v>917</v>
+        <v>908</v>
       </c>
       <c r="C500" s="8" t="s">
-        <v>921</v>
+        <v>912</v>
       </c>
       <c r="D500" s="7" t="s">
         <v>32</v>
@@ -25946,10 +25971,10 @@
         <v>493</v>
       </c>
       <c r="B501" s="23" t="s">
-        <v>917</v>
+        <v>908</v>
       </c>
       <c r="C501" s="8" t="s">
-        <v>922</v>
+        <v>913</v>
       </c>
       <c r="D501" s="7" t="s">
         <v>32</v>
@@ -25982,10 +26007,10 @@
         <v>494</v>
       </c>
       <c r="B502" s="23" t="s">
-        <v>917</v>
+        <v>908</v>
       </c>
       <c r="C502" s="8" t="s">
-        <v>923</v>
+        <v>914</v>
       </c>
       <c r="D502" s="7" t="s">
         <v>32</v>
@@ -26018,10 +26043,10 @@
         <v>495</v>
       </c>
       <c r="B503" s="23" t="s">
-        <v>917</v>
+        <v>908</v>
       </c>
       <c r="C503" s="8" t="s">
-        <v>924</v>
+        <v>915</v>
       </c>
       <c r="D503" s="7" t="s">
         <v>32</v>
@@ -26054,10 +26079,10 @@
         <v>496</v>
       </c>
       <c r="B504" s="23" t="s">
-        <v>917</v>
+        <v>908</v>
       </c>
       <c r="C504" s="8" t="s">
-        <v>925</v>
+        <v>916</v>
       </c>
       <c r="D504" s="7" t="s">
         <v>32</v>
@@ -26090,10 +26115,10 @@
         <v>497</v>
       </c>
       <c r="B505" s="23" t="s">
+        <v>908</v>
+      </c>
+      <c r="C505" s="8" t="s">
         <v>917</v>
-      </c>
-      <c r="C505" s="8" t="s">
-        <v>926</v>
       </c>
       <c r="D505" s="7" t="s">
         <v>32</v>
@@ -26126,10 +26151,10 @@
         <v>498</v>
       </c>
       <c r="B506" s="23" t="s">
-        <v>917</v>
+        <v>908</v>
       </c>
       <c r="C506" s="8" t="s">
-        <v>927</v>
+        <v>918</v>
       </c>
       <c r="D506" s="7" t="s">
         <v>32</v>
@@ -26162,10 +26187,10 @@
         <v>499</v>
       </c>
       <c r="B507" s="23" t="s">
-        <v>917</v>
+        <v>908</v>
       </c>
       <c r="C507" s="8" t="s">
-        <v>928</v>
+        <v>919</v>
       </c>
       <c r="D507" s="7" t="s">
         <v>32</v>
@@ -26198,10 +26223,10 @@
         <v>500</v>
       </c>
       <c r="B508" s="23" t="s">
-        <v>917</v>
+        <v>908</v>
       </c>
       <c r="C508" s="8" t="s">
-        <v>929</v>
+        <v>920</v>
       </c>
       <c r="D508" s="7" t="s">
         <v>32</v>
@@ -26234,10 +26259,10 @@
         <v>501</v>
       </c>
       <c r="B509" s="23" t="s">
-        <v>917</v>
+        <v>908</v>
       </c>
       <c r="C509" s="8" t="s">
-        <v>930</v>
+        <v>921</v>
       </c>
       <c r="D509" s="7" t="s">
         <v>32</v>
@@ -26270,10 +26295,10 @@
         <v>502</v>
       </c>
       <c r="B510" s="23" t="s">
-        <v>917</v>
+        <v>908</v>
       </c>
       <c r="C510" s="8" t="s">
-        <v>931</v>
+        <v>922</v>
       </c>
       <c r="D510" s="7" t="s">
         <v>32</v>
@@ -26306,10 +26331,10 @@
         <v>503</v>
       </c>
       <c r="B511" s="23" t="s">
-        <v>917</v>
+        <v>908</v>
       </c>
       <c r="C511" s="8" t="s">
-        <v>932</v>
+        <v>923</v>
       </c>
       <c r="D511" s="7" t="s">
         <v>32</v>
@@ -26342,10 +26367,10 @@
         <v>504</v>
       </c>
       <c r="B512" s="23" t="s">
-        <v>917</v>
+        <v>908</v>
       </c>
       <c r="C512" s="8" t="s">
-        <v>933</v>
+        <v>924</v>
       </c>
       <c r="D512" s="7" t="s">
         <v>32</v>
@@ -26378,10 +26403,10 @@
         <v>505</v>
       </c>
       <c r="B513" s="23" t="s">
-        <v>917</v>
+        <v>908</v>
       </c>
       <c r="C513" s="8" t="s">
-        <v>934</v>
+        <v>925</v>
       </c>
       <c r="D513" s="7" t="s">
         <v>32</v>
@@ -26414,10 +26439,10 @@
         <v>506</v>
       </c>
       <c r="B514" s="23" t="s">
-        <v>917</v>
+        <v>908</v>
       </c>
       <c r="C514" s="8" t="s">
-        <v>935</v>
+        <v>926</v>
       </c>
       <c r="D514" s="7" t="s">
         <v>32</v>
@@ -26450,10 +26475,10 @@
         <v>507</v>
       </c>
       <c r="B515" s="23" t="s">
-        <v>917</v>
+        <v>908</v>
       </c>
       <c r="C515" s="8" t="s">
-        <v>936</v>
+        <v>927</v>
       </c>
       <c r="D515" s="7" t="s">
         <v>32</v>
@@ -26486,10 +26511,10 @@
         <v>508</v>
       </c>
       <c r="B516" s="23" t="s">
-        <v>917</v>
+        <v>908</v>
       </c>
       <c r="C516" s="8" t="s">
-        <v>937</v>
+        <v>928</v>
       </c>
       <c r="D516" s="7" t="s">
         <v>32</v>
@@ -26501,7 +26526,7 @@
         <v>1</v>
       </c>
       <c r="H516" s="13" t="s">
-        <v>938</v>
+        <v>929</v>
       </c>
       <c r="M516" s="9" t="str" cm="1">
         <f t="array" ref="M516">PAGE_NAME(B516)</f>
@@ -26525,10 +26550,10 @@
         <v>509</v>
       </c>
       <c r="B517" s="23" t="s">
-        <v>917</v>
+        <v>908</v>
       </c>
       <c r="C517" s="8" t="s">
-        <v>939</v>
+        <v>930</v>
       </c>
       <c r="D517" s="7" t="s">
         <v>41</v>
@@ -26540,7 +26565,7 @@
         <v>1</v>
       </c>
       <c r="H517" s="13" t="s">
-        <v>940</v>
+        <v>931</v>
       </c>
       <c r="M517" s="9" t="str" cm="1">
         <f t="array" ref="M517">PAGE_NAME(B517)</f>
@@ -26564,10 +26589,10 @@
         <v>510</v>
       </c>
       <c r="B518" s="23" t="s">
-        <v>917</v>
+        <v>908</v>
       </c>
       <c r="C518" s="8" t="s">
-        <v>941</v>
+        <v>932</v>
       </c>
       <c r="D518" s="7" t="s">
         <v>37</v>
@@ -26600,10 +26625,10 @@
         <v>511</v>
       </c>
       <c r="B519" s="23" t="s">
-        <v>942</v>
+        <v>933</v>
       </c>
       <c r="C519" s="8" t="s">
-        <v>943</v>
+        <v>934</v>
       </c>
       <c r="D519" s="7" t="s">
         <v>32</v>
@@ -26615,7 +26640,7 @@
         <v>1</v>
       </c>
       <c r="H519" s="13" t="s">
-        <v>944</v>
+        <v>935</v>
       </c>
       <c r="M519" s="9" t="str" cm="1">
         <f t="array" ref="M519">PAGE_NAME(B519)</f>
@@ -26639,10 +26664,10 @@
         <v>512</v>
       </c>
       <c r="B520" s="23" t="s">
-        <v>942</v>
+        <v>933</v>
       </c>
       <c r="C520" s="8" t="s">
-        <v>945</v>
+        <v>936</v>
       </c>
       <c r="D520" s="7" t="s">
         <v>41</v>
@@ -26654,7 +26679,7 @@
         <v>1</v>
       </c>
       <c r="H520" s="13" t="s">
-        <v>944</v>
+        <v>935</v>
       </c>
       <c r="M520" s="9" t="str" cm="1">
         <f t="array" ref="M520">PAGE_NAME(B520)</f>
@@ -26678,10 +26703,10 @@
         <v>513</v>
       </c>
       <c r="B521" s="23" t="s">
-        <v>946</v>
+        <v>937</v>
       </c>
       <c r="C521" s="8" t="s">
-        <v>947</v>
+        <v>938</v>
       </c>
       <c r="D521" s="7" t="s">
         <v>87</v>
@@ -26717,10 +26742,10 @@
         <v>514</v>
       </c>
       <c r="B522" s="23" t="s">
-        <v>948</v>
+        <v>939</v>
       </c>
       <c r="C522" s="8" t="s">
-        <v>949</v>
+        <v>940</v>
       </c>
       <c r="D522" s="7" t="s">
         <v>41</v>
@@ -26753,10 +26778,10 @@
         <v>515</v>
       </c>
       <c r="B523" s="23" t="s">
-        <v>948</v>
+        <v>939</v>
       </c>
       <c r="C523" s="8" t="s">
-        <v>950</v>
+        <v>941</v>
       </c>
       <c r="D523" s="7" t="s">
         <v>37</v>
@@ -26789,10 +26814,10 @@
         <v>516</v>
       </c>
       <c r="B524" s="53" t="s">
-        <v>948</v>
+        <v>939</v>
       </c>
       <c r="C524" s="8" t="s">
-        <v>951</v>
+        <v>942</v>
       </c>
       <c r="D524" s="7" t="s">
         <v>87</v>
@@ -26804,7 +26829,7 @@
         <v>1</v>
       </c>
       <c r="H524" s="13" t="s">
-        <v>908</v>
+        <v>899</v>
       </c>
       <c r="M524" s="9" t="str" cm="1">
         <f t="array" ref="M524">PAGE_NAME(B524)</f>
@@ -26823,7 +26848,7 @@
         <v>Server</v>
       </c>
       <c r="U524" s="13" t="s">
-        <v>899</v>
+        <v>890</v>
       </c>
     </row>
     <row r="525" spans="1:21" ht="85" x14ac:dyDescent="0.2">
@@ -26831,10 +26856,10 @@
         <v>517</v>
       </c>
       <c r="B525" s="23" t="s">
-        <v>948</v>
+        <v>939</v>
       </c>
       <c r="C525" s="8" t="s">
-        <v>952</v>
+        <v>943</v>
       </c>
       <c r="D525" s="7" t="s">
         <v>87</v>
@@ -26846,7 +26871,7 @@
         <v>1</v>
       </c>
       <c r="H525" s="13" t="s">
-        <v>908</v>
+        <v>899</v>
       </c>
       <c r="M525" s="9" t="str" cm="1">
         <f t="array" ref="M525">PAGE_NAME(B525)</f>
@@ -26865,7 +26890,7 @@
         <v>Client</v>
       </c>
       <c r="U525" s="13" t="s">
-        <v>899</v>
+        <v>890</v>
       </c>
     </row>
     <row r="526" spans="1:21" ht="119" x14ac:dyDescent="0.2">
@@ -26873,10 +26898,10 @@
         <v>518</v>
       </c>
       <c r="B526" s="23" t="s">
-        <v>948</v>
+        <v>939</v>
       </c>
       <c r="C526" s="8" t="s">
-        <v>953</v>
+        <v>944</v>
       </c>
       <c r="D526" s="7" t="s">
         <v>87</v>
@@ -26888,7 +26913,7 @@
         <v>1</v>
       </c>
       <c r="H526" s="13" t="s">
-        <v>911</v>
+        <v>902</v>
       </c>
       <c r="M526" s="9" t="str" cm="1">
         <f t="array" ref="M526">PAGE_NAME(B526)</f>
@@ -26907,7 +26932,7 @@
         <v>Server</v>
       </c>
       <c r="U526" s="13" t="s">
-        <v>899</v>
+        <v>890</v>
       </c>
     </row>
     <row r="527" spans="1:21" ht="85" x14ac:dyDescent="0.2">
@@ -26915,10 +26940,10 @@
         <v>519</v>
       </c>
       <c r="B527" s="23" t="s">
-        <v>948</v>
+        <v>939</v>
       </c>
       <c r="C527" s="8" t="s">
-        <v>954</v>
+        <v>945</v>
       </c>
       <c r="D527" s="7" t="s">
         <v>87</v>
@@ -26930,7 +26955,7 @@
         <v>1</v>
       </c>
       <c r="H527" s="13" t="s">
-        <v>908</v>
+        <v>899</v>
       </c>
       <c r="M527" s="9" t="str" cm="1">
         <f t="array" ref="M527">PAGE_NAME(B527)</f>
@@ -26949,7 +26974,7 @@
         <v>Client</v>
       </c>
       <c r="U527" s="13" t="s">
-        <v>899</v>
+        <v>890</v>
       </c>
     </row>
     <row r="528" spans="1:21" ht="85" x14ac:dyDescent="0.2">
@@ -26957,10 +26982,10 @@
         <v>520</v>
       </c>
       <c r="B528" s="23" t="s">
-        <v>948</v>
+        <v>939</v>
       </c>
       <c r="C528" s="8" t="s">
-        <v>955</v>
+        <v>946</v>
       </c>
       <c r="D528" s="7" t="s">
         <v>87</v>
@@ -26972,7 +26997,7 @@
         <v>1</v>
       </c>
       <c r="H528" s="13" t="s">
-        <v>914</v>
+        <v>905</v>
       </c>
       <c r="M528" s="9" t="str" cm="1">
         <f t="array" ref="M528">PAGE_NAME(B528)</f>
@@ -26991,7 +27016,7 @@
         <v>Server</v>
       </c>
       <c r="U528" s="13" t="s">
-        <v>899</v>
+        <v>890</v>
       </c>
     </row>
     <row r="529" spans="1:21" ht="85" x14ac:dyDescent="0.2">
@@ -26999,10 +27024,10 @@
         <v>521</v>
       </c>
       <c r="B529" s="53" t="s">
-        <v>948</v>
+        <v>939</v>
       </c>
       <c r="C529" s="8" t="s">
-        <v>956</v>
+        <v>947</v>
       </c>
       <c r="D529" s="7" t="s">
         <v>87</v>
@@ -27014,7 +27039,7 @@
         <v>1</v>
       </c>
       <c r="H529" s="13" t="s">
-        <v>914</v>
+        <v>905</v>
       </c>
       <c r="M529" s="9" t="str" cm="1">
         <f t="array" ref="M529">PAGE_NAME(B529)</f>
@@ -27033,7 +27058,7 @@
         <v>Client</v>
       </c>
       <c r="U529" s="13" t="s">
-        <v>899</v>
+        <v>890</v>
       </c>
     </row>
     <row r="530" spans="1:21" ht="102" x14ac:dyDescent="0.2">
@@ -27041,10 +27066,10 @@
         <v>522</v>
       </c>
       <c r="B530" s="23" t="s">
+        <v>939</v>
+      </c>
+      <c r="C530" s="8" t="s">
         <v>948</v>
-      </c>
-      <c r="C530" s="8" t="s">
-        <v>957</v>
       </c>
       <c r="D530" s="7" t="s">
         <v>37</v>
@@ -27072,7 +27097,7 @@
         <v/>
       </c>
       <c r="U530" s="13" t="s">
-        <v>958</v>
+        <v>949</v>
       </c>
     </row>
     <row r="531" spans="1:21" ht="68" x14ac:dyDescent="0.2">
@@ -27080,10 +27105,10 @@
         <v>523</v>
       </c>
       <c r="B531" s="23" t="s">
-        <v>959</v>
+        <v>950</v>
       </c>
       <c r="C531" s="8" t="s">
-        <v>960</v>
+        <v>951</v>
       </c>
       <c r="D531" s="7" t="s">
         <v>41</v>
@@ -27116,10 +27141,10 @@
         <v>524</v>
       </c>
       <c r="B532" s="23" t="s">
-        <v>959</v>
+        <v>950</v>
       </c>
       <c r="C532" s="8" t="s">
-        <v>961</v>
+        <v>952</v>
       </c>
       <c r="D532" s="7" t="s">
         <v>87</v>
@@ -27131,7 +27156,7 @@
         <v>1</v>
       </c>
       <c r="H532" s="13" t="s">
-        <v>962</v>
+        <v>953</v>
       </c>
       <c r="M532" s="9" t="str" cm="1">
         <f t="array" ref="M532">PAGE_NAME(B532)</f>
@@ -27150,7 +27175,7 @@
         <v>Server</v>
       </c>
       <c r="U532" s="13" t="s">
-        <v>899</v>
+        <v>890</v>
       </c>
     </row>
     <row r="533" spans="1:21" ht="51" x14ac:dyDescent="0.2">
@@ -27158,10 +27183,10 @@
         <v>525</v>
       </c>
       <c r="B533" s="23" t="s">
-        <v>959</v>
+        <v>950</v>
       </c>
       <c r="C533" s="8" t="s">
-        <v>963</v>
+        <v>954</v>
       </c>
       <c r="D533" s="7" t="s">
         <v>87</v>
@@ -27189,7 +27214,7 @@
         <v>Client</v>
       </c>
       <c r="U533" s="13" t="s">
-        <v>899</v>
+        <v>890</v>
       </c>
     </row>
     <row r="534" spans="1:21" ht="51" x14ac:dyDescent="0.2">
@@ -27197,10 +27222,10 @@
         <v>526</v>
       </c>
       <c r="B534" s="23" t="s">
-        <v>959</v>
+        <v>950</v>
       </c>
       <c r="C534" s="8" t="s">
-        <v>964</v>
+        <v>955</v>
       </c>
       <c r="D534" s="7" t="s">
         <v>41</v>
@@ -27233,10 +27258,10 @@
         <v>527</v>
       </c>
       <c r="B535" s="23" t="s">
-        <v>965</v>
+        <v>956</v>
       </c>
       <c r="C535" s="8" t="s">
-        <v>966</v>
+        <v>957</v>
       </c>
       <c r="D535" s="7" t="s">
         <v>37</v>
@@ -27264,7 +27289,7 @@
         <v>Client</v>
       </c>
       <c r="U535" s="13" t="s">
-        <v>967</v>
+        <v>958</v>
       </c>
     </row>
     <row r="536" spans="1:21" ht="34" x14ac:dyDescent="0.2">
@@ -27272,10 +27297,10 @@
         <v>528</v>
       </c>
       <c r="B536" s="23" t="s">
-        <v>968</v>
+        <v>959</v>
       </c>
       <c r="C536" s="8" t="s">
-        <v>969</v>
+        <v>960</v>
       </c>
       <c r="D536" s="7" t="s">
         <v>41</v>
@@ -27308,10 +27333,10 @@
         <v>529</v>
       </c>
       <c r="B537" s="23" t="s">
-        <v>968</v>
+        <v>959</v>
       </c>
       <c r="C537" s="8" t="s">
-        <v>970</v>
+        <v>961</v>
       </c>
       <c r="D537" s="7" t="s">
         <v>41</v>
@@ -27344,10 +27369,10 @@
         <v>530</v>
       </c>
       <c r="B538" s="23" t="s">
-        <v>968</v>
+        <v>959</v>
       </c>
       <c r="C538" s="8" t="s">
-        <v>971</v>
+        <v>962</v>
       </c>
       <c r="D538" s="7" t="s">
         <v>41</v>
@@ -27380,10 +27405,10 @@
         <v>531</v>
       </c>
       <c r="B539" s="23" t="s">
-        <v>968</v>
+        <v>959</v>
       </c>
       <c r="C539" s="8" t="s">
-        <v>972</v>
+        <v>963</v>
       </c>
       <c r="D539" s="7" t="s">
         <v>41</v>
@@ -27416,10 +27441,10 @@
         <v>532</v>
       </c>
       <c r="B540" s="23" t="s">
-        <v>973</v>
+        <v>964</v>
       </c>
       <c r="C540" s="8" t="s">
-        <v>974</v>
+        <v>965</v>
       </c>
       <c r="D540" s="7" t="s">
         <v>37</v>
@@ -27447,7 +27472,7 @@
         <v>Server</v>
       </c>
       <c r="U540" s="13" t="s">
-        <v>975</v>
+        <v>966</v>
       </c>
     </row>
     <row r="541" spans="1:21" ht="34" x14ac:dyDescent="0.2">
@@ -27455,10 +27480,10 @@
         <v>533</v>
       </c>
       <c r="B541" s="23" t="s">
-        <v>976</v>
+        <v>967</v>
       </c>
       <c r="C541" s="8" t="s">
-        <v>977</v>
+        <v>968</v>
       </c>
       <c r="D541" s="7" t="s">
         <v>32</v>
@@ -27491,10 +27516,10 @@
         <v>534</v>
       </c>
       <c r="B542" s="23" t="s">
-        <v>976</v>
+        <v>967</v>
       </c>
       <c r="C542" s="8" t="s">
-        <v>978</v>
+        <v>969</v>
       </c>
       <c r="D542" s="7" t="s">
         <v>32</v>
@@ -27527,10 +27552,10 @@
         <v>535</v>
       </c>
       <c r="B543" s="23" t="s">
-        <v>976</v>
+        <v>967</v>
       </c>
       <c r="C543" s="8" t="s">
-        <v>979</v>
+        <v>970</v>
       </c>
       <c r="D543" s="7" t="s">
         <v>32</v>
@@ -27563,10 +27588,10 @@
         <v>536</v>
       </c>
       <c r="B544" s="23" t="s">
-        <v>976</v>
+        <v>967</v>
       </c>
       <c r="C544" s="8" t="s">
-        <v>980</v>
+        <v>971</v>
       </c>
       <c r="D544" s="7" t="s">
         <v>32</v>
@@ -27599,10 +27624,10 @@
         <v>537</v>
       </c>
       <c r="B545" s="23" t="s">
-        <v>976</v>
+        <v>967</v>
       </c>
       <c r="C545" s="8" t="s">
-        <v>981</v>
+        <v>972</v>
       </c>
       <c r="D545" s="7" t="s">
         <v>32</v>
@@ -27635,10 +27660,10 @@
         <v>538</v>
       </c>
       <c r="B546" s="23" t="s">
-        <v>976</v>
+        <v>967</v>
       </c>
       <c r="C546" s="8" t="s">
-        <v>982</v>
+        <v>973</v>
       </c>
       <c r="D546" s="7" t="s">
         <v>32</v>
@@ -27671,10 +27696,10 @@
         <v>539</v>
       </c>
       <c r="B547" s="23" t="s">
-        <v>976</v>
+        <v>967</v>
       </c>
       <c r="C547" s="8" t="s">
-        <v>983</v>
+        <v>974</v>
       </c>
       <c r="D547" s="7" t="s">
         <v>32</v>
@@ -27707,10 +27732,10 @@
         <v>540</v>
       </c>
       <c r="B548" s="23" t="s">
-        <v>976</v>
+        <v>967</v>
       </c>
       <c r="C548" s="8" t="s">
-        <v>984</v>
+        <v>975</v>
       </c>
       <c r="D548" s="7" t="s">
         <v>32</v>
@@ -27743,10 +27768,10 @@
         <v>541</v>
       </c>
       <c r="B549" s="23" t="s">
+        <v>967</v>
+      </c>
+      <c r="C549" s="8" t="s">
         <v>976</v>
-      </c>
-      <c r="C549" s="8" t="s">
-        <v>985</v>
       </c>
       <c r="D549" s="7" t="s">
         <v>37</v>
@@ -27779,10 +27804,10 @@
         <v>542</v>
       </c>
       <c r="B550" s="23" t="s">
-        <v>976</v>
+        <v>967</v>
       </c>
       <c r="C550" s="8" t="s">
-        <v>986</v>
+        <v>977</v>
       </c>
       <c r="D550" s="7" t="s">
         <v>37</v>
@@ -27815,10 +27840,10 @@
         <v>543</v>
       </c>
       <c r="B551" s="23" t="s">
-        <v>976</v>
+        <v>967</v>
       </c>
       <c r="C551" s="8" t="s">
-        <v>987</v>
+        <v>978</v>
       </c>
       <c r="D551" s="7" t="s">
         <v>32</v>
@@ -27830,7 +27855,7 @@
         <v>1</v>
       </c>
       <c r="H551" s="13" t="s">
-        <v>988</v>
+        <v>979</v>
       </c>
       <c r="M551" s="9" t="str" cm="1">
         <f t="array" ref="M551">PAGE_NAME(B551)</f>
@@ -27854,10 +27879,10 @@
         <v>544</v>
       </c>
       <c r="B552" s="23" t="s">
-        <v>976</v>
+        <v>967</v>
       </c>
       <c r="C552" s="8" t="s">
-        <v>989</v>
+        <v>980</v>
       </c>
       <c r="D552" s="7" t="s">
         <v>41</v>
@@ -27890,10 +27915,10 @@
         <v>545</v>
       </c>
       <c r="B553" s="23" t="s">
-        <v>976</v>
+        <v>967</v>
       </c>
       <c r="C553" s="8" t="s">
-        <v>990</v>
+        <v>981</v>
       </c>
       <c r="D553" s="7" t="s">
         <v>41</v>
@@ -27926,10 +27951,10 @@
         <v>546</v>
       </c>
       <c r="B554" s="23" t="s">
-        <v>976</v>
+        <v>967</v>
       </c>
       <c r="C554" s="8" t="s">
-        <v>991</v>
+        <v>982</v>
       </c>
       <c r="D554" s="7" t="s">
         <v>41</v>
@@ -27962,10 +27987,10 @@
         <v>547</v>
       </c>
       <c r="B555" s="23" t="s">
-        <v>976</v>
+        <v>967</v>
       </c>
       <c r="C555" s="8" t="s">
-        <v>992</v>
+        <v>983</v>
       </c>
       <c r="D555" s="7" t="s">
         <v>41</v>
@@ -27998,10 +28023,10 @@
         <v>548</v>
       </c>
       <c r="B556" s="23" t="s">
-        <v>993</v>
+        <v>984</v>
       </c>
       <c r="C556" s="8" t="s">
-        <v>994</v>
+        <v>985</v>
       </c>
       <c r="D556" s="7" t="s">
         <v>37</v>
@@ -28034,10 +28059,10 @@
         <v>549</v>
       </c>
       <c r="B557" s="23" t="s">
-        <v>993</v>
+        <v>984</v>
       </c>
       <c r="C557" s="8" t="s">
-        <v>995</v>
+        <v>986</v>
       </c>
       <c r="D557" s="7" t="s">
         <v>37</v>
@@ -28049,7 +28074,7 @@
         <v>1</v>
       </c>
       <c r="H557" s="13" t="s">
-        <v>996</v>
+        <v>987</v>
       </c>
       <c r="M557" s="9" t="str" cm="1">
         <f t="array" ref="M557">PAGE_NAME(B557)</f>
@@ -28073,10 +28098,10 @@
         <v>550</v>
       </c>
       <c r="B558" s="23" t="s">
-        <v>997</v>
+        <v>988</v>
       </c>
       <c r="C558" s="8" t="s">
-        <v>998</v>
+        <v>989</v>
       </c>
       <c r="D558" s="7" t="s">
         <v>32</v>
@@ -28109,10 +28134,10 @@
         <v>551</v>
       </c>
       <c r="B559" s="23" t="s">
-        <v>997</v>
+        <v>988</v>
       </c>
       <c r="C559" s="8" t="s">
-        <v>998</v>
+        <v>989</v>
       </c>
       <c r="D559" s="7" t="s">
         <v>32</v>
@@ -28145,10 +28170,10 @@
         <v>552</v>
       </c>
       <c r="B560" s="23" t="s">
-        <v>997</v>
+        <v>988</v>
       </c>
       <c r="C560" s="8" t="s">
-        <v>999</v>
+        <v>990</v>
       </c>
       <c r="D560" s="7" t="s">
         <v>37</v>
@@ -28181,10 +28206,10 @@
         <v>553</v>
       </c>
       <c r="B561" s="23" t="s">
-        <v>997</v>
+        <v>988</v>
       </c>
       <c r="C561" s="8" t="s">
-        <v>999</v>
+        <v>990</v>
       </c>
       <c r="D561" s="7" t="s">
         <v>37</v>
@@ -28217,10 +28242,10 @@
         <v>554</v>
       </c>
       <c r="B562" s="23" t="s">
-        <v>997</v>
+        <v>988</v>
       </c>
       <c r="C562" s="8" t="s">
-        <v>1000</v>
+        <v>991</v>
       </c>
       <c r="D562" s="7" t="s">
         <v>37</v>
@@ -28253,10 +28278,10 @@
         <v>555</v>
       </c>
       <c r="B563" s="23" t="s">
-        <v>997</v>
+        <v>988</v>
       </c>
       <c r="C563" s="8" t="s">
-        <v>1000</v>
+        <v>991</v>
       </c>
       <c r="D563" s="7" t="s">
         <v>37</v>
@@ -28289,10 +28314,10 @@
         <v>556</v>
       </c>
       <c r="B564" s="23" t="s">
-        <v>997</v>
+        <v>988</v>
       </c>
       <c r="C564" s="8" t="s">
-        <v>1001</v>
+        <v>992</v>
       </c>
       <c r="D564" s="7" t="s">
         <v>37</v>
@@ -28325,10 +28350,10 @@
         <v>557</v>
       </c>
       <c r="B565" s="23" t="s">
-        <v>997</v>
+        <v>988</v>
       </c>
       <c r="C565" s="8" t="s">
-        <v>1001</v>
+        <v>992</v>
       </c>
       <c r="D565" s="7" t="s">
         <v>37</v>
@@ -28361,10 +28386,10 @@
         <v>558</v>
       </c>
       <c r="B566" s="23" t="s">
-        <v>997</v>
+        <v>988</v>
       </c>
       <c r="C566" s="8" t="s">
-        <v>1002</v>
+        <v>993</v>
       </c>
       <c r="D566" s="7" t="s">
         <v>32</v>
@@ -28397,10 +28422,10 @@
         <v>559</v>
       </c>
       <c r="B567" s="23" t="s">
-        <v>997</v>
+        <v>988</v>
       </c>
       <c r="C567" s="8" t="s">
-        <v>1002</v>
+        <v>993</v>
       </c>
       <c r="D567" s="7" t="s">
         <v>32</v>
@@ -28433,10 +28458,10 @@
         <v>560</v>
       </c>
       <c r="B568" s="23" t="s">
-        <v>997</v>
+        <v>988</v>
       </c>
       <c r="C568" s="8" t="s">
-        <v>1003</v>
+        <v>994</v>
       </c>
       <c r="D568" s="7" t="s">
         <v>37</v>
@@ -28469,10 +28494,10 @@
         <v>561</v>
       </c>
       <c r="B569" s="23" t="s">
-        <v>997</v>
+        <v>988</v>
       </c>
       <c r="C569" s="8" t="s">
-        <v>1003</v>
+        <v>994</v>
       </c>
       <c r="D569" s="7" t="s">
         <v>37</v>
@@ -28505,10 +28530,10 @@
         <v>562</v>
       </c>
       <c r="B570" s="23" t="s">
-        <v>997</v>
+        <v>988</v>
       </c>
       <c r="C570" s="8" t="s">
-        <v>1004</v>
+        <v>995</v>
       </c>
       <c r="D570" s="7" t="s">
         <v>32</v>
@@ -28541,10 +28566,10 @@
         <v>563</v>
       </c>
       <c r="B571" s="23" t="s">
-        <v>997</v>
+        <v>988</v>
       </c>
       <c r="C571" s="8" t="s">
-        <v>1004</v>
+        <v>995</v>
       </c>
       <c r="D571" s="7" t="s">
         <v>32</v>
@@ -28577,10 +28602,10 @@
         <v>564</v>
       </c>
       <c r="B572" s="23" t="s">
-        <v>997</v>
+        <v>988</v>
       </c>
       <c r="C572" s="8" t="s">
-        <v>1005</v>
+        <v>996</v>
       </c>
       <c r="D572" s="7" t="s">
         <v>32</v>
@@ -28613,10 +28638,10 @@
         <v>565</v>
       </c>
       <c r="B573" s="23" t="s">
-        <v>997</v>
+        <v>988</v>
       </c>
       <c r="C573" s="8" t="s">
-        <v>1005</v>
+        <v>996</v>
       </c>
       <c r="D573" s="7" t="s">
         <v>32</v>
@@ -28649,10 +28674,10 @@
         <v>566</v>
       </c>
       <c r="B574" s="23" t="s">
+        <v>988</v>
+      </c>
+      <c r="C574" s="8" t="s">
         <v>997</v>
-      </c>
-      <c r="C574" s="8" t="s">
-        <v>1006</v>
       </c>
       <c r="D574" s="7" t="s">
         <v>37</v>
@@ -28685,10 +28710,10 @@
         <v>567</v>
       </c>
       <c r="B575" s="23" t="s">
+        <v>988</v>
+      </c>
+      <c r="C575" s="8" t="s">
         <v>997</v>
-      </c>
-      <c r="C575" s="8" t="s">
-        <v>1006</v>
       </c>
       <c r="D575" s="7" t="s">
         <v>37</v>
@@ -28721,10 +28746,10 @@
         <v>568</v>
       </c>
       <c r="B576" s="23" t="s">
-        <v>997</v>
+        <v>988</v>
       </c>
       <c r="C576" s="8" t="s">
-        <v>1007</v>
+        <v>998</v>
       </c>
       <c r="D576" s="7" t="s">
         <v>32</v>
@@ -28757,10 +28782,10 @@
         <v>569</v>
       </c>
       <c r="B577" s="23" t="s">
-        <v>997</v>
+        <v>988</v>
       </c>
       <c r="C577" s="8" t="s">
-        <v>1007</v>
+        <v>998</v>
       </c>
       <c r="D577" s="7" t="s">
         <v>32</v>
@@ -28793,10 +28818,10 @@
         <v>570</v>
       </c>
       <c r="B578" s="23" t="s">
-        <v>997</v>
+        <v>988</v>
       </c>
       <c r="C578" s="8" t="s">
-        <v>1008</v>
+        <v>999</v>
       </c>
       <c r="D578" s="7" t="s">
         <v>32</v>
@@ -28829,10 +28854,10 @@
         <v>571</v>
       </c>
       <c r="B579" s="23" t="s">
-        <v>997</v>
+        <v>988</v>
       </c>
       <c r="C579" s="8" t="s">
-        <v>1008</v>
+        <v>999</v>
       </c>
       <c r="D579" s="7" t="s">
         <v>32</v>
@@ -28865,10 +28890,10 @@
         <v>572</v>
       </c>
       <c r="B580" s="23" t="s">
-        <v>997</v>
+        <v>988</v>
       </c>
       <c r="C580" s="8" t="s">
-        <v>1009</v>
+        <v>1000</v>
       </c>
       <c r="D580" s="7" t="s">
         <v>32</v>
@@ -28901,10 +28926,10 @@
         <v>573</v>
       </c>
       <c r="B581" s="23" t="s">
-        <v>997</v>
+        <v>988</v>
       </c>
       <c r="C581" s="8" t="s">
-        <v>1009</v>
+        <v>1000</v>
       </c>
       <c r="D581" s="7" t="s">
         <v>32</v>
@@ -28937,10 +28962,10 @@
         <v>574</v>
       </c>
       <c r="B582" s="23" t="s">
-        <v>997</v>
+        <v>988</v>
       </c>
       <c r="C582" s="8" t="s">
-        <v>1010</v>
+        <v>1001</v>
       </c>
       <c r="D582" s="7" t="s">
         <v>37</v>
@@ -28973,10 +28998,10 @@
         <v>575</v>
       </c>
       <c r="B583" s="23" t="s">
-        <v>997</v>
+        <v>988</v>
       </c>
       <c r="C583" s="8" t="s">
-        <v>1010</v>
+        <v>1001</v>
       </c>
       <c r="D583" s="7" t="s">
         <v>37</v>
@@ -29009,10 +29034,10 @@
         <v>576</v>
       </c>
       <c r="B584" s="23" t="s">
-        <v>997</v>
+        <v>988</v>
       </c>
       <c r="C584" s="8" t="s">
-        <v>1011</v>
+        <v>1002</v>
       </c>
       <c r="D584" s="7" t="s">
         <v>37</v>
@@ -29045,10 +29070,10 @@
         <v>577</v>
       </c>
       <c r="B585" s="23" t="s">
-        <v>997</v>
+        <v>988</v>
       </c>
       <c r="C585" s="8" t="s">
-        <v>1012</v>
+        <v>1003</v>
       </c>
       <c r="D585" s="7" t="s">
         <v>37</v>
@@ -29081,10 +29106,10 @@
         <v>578</v>
       </c>
       <c r="B586" s="23" t="s">
-        <v>997</v>
+        <v>988</v>
       </c>
       <c r="C586" s="8" t="s">
-        <v>1013</v>
+        <v>1004</v>
       </c>
       <c r="D586" s="7" t="s">
         <v>41</v>
@@ -29117,10 +29142,10 @@
         <v>579</v>
       </c>
       <c r="B587" s="23" t="s">
-        <v>997</v>
+        <v>988</v>
       </c>
       <c r="C587" s="8" t="s">
-        <v>1013</v>
+        <v>1004</v>
       </c>
       <c r="D587" s="7" t="s">
         <v>41</v>
@@ -29153,10 +29178,10 @@
         <v>580</v>
       </c>
       <c r="B588" s="23" t="s">
-        <v>997</v>
+        <v>988</v>
       </c>
       <c r="C588" s="8" t="s">
-        <v>1014</v>
+        <v>1005</v>
       </c>
       <c r="D588" s="7" t="s">
         <v>41</v>
@@ -29189,10 +29214,10 @@
         <v>581</v>
       </c>
       <c r="B589" s="23" t="s">
-        <v>997</v>
+        <v>988</v>
       </c>
       <c r="C589" s="8" t="s">
-        <v>1014</v>
+        <v>1005</v>
       </c>
       <c r="D589" s="7" t="s">
         <v>41</v>
@@ -29225,10 +29250,10 @@
         <v>582</v>
       </c>
       <c r="B590" s="39" t="s">
-        <v>1015</v>
+        <v>1006</v>
       </c>
       <c r="C590" s="8" t="s">
-        <v>1016</v>
+        <v>1007</v>
       </c>
       <c r="D590" s="7" t="s">
         <v>87</v>
@@ -29240,7 +29265,7 @@
         <v>1</v>
       </c>
       <c r="H590" s="13" t="s">
-        <v>1017</v>
+        <v>1008</v>
       </c>
       <c r="M590" s="9" t="str" cm="1">
         <f t="array" ref="M590">PAGE_NAME(B590)</f>
@@ -29257,10 +29282,10 @@
         <v>583</v>
       </c>
       <c r="B591" s="39" t="s">
-        <v>1015</v>
+        <v>1006</v>
       </c>
       <c r="C591" s="8" t="s">
-        <v>1016</v>
+        <v>1007</v>
       </c>
       <c r="D591" s="7" t="s">
         <v>87</v>
@@ -29272,7 +29297,7 @@
         <v>1</v>
       </c>
       <c r="H591" s="13" t="s">
-        <v>1017</v>
+        <v>1008</v>
       </c>
       <c r="M591" s="9" t="str" cm="1">
         <f t="array" ref="M591">PAGE_NAME(B591)</f>
@@ -29289,10 +29314,10 @@
         <v>584</v>
       </c>
       <c r="B592" s="11" t="s">
-        <v>1018</v>
+        <v>1009</v>
       </c>
       <c r="C592" s="8" t="s">
-        <v>1019</v>
+        <v>1010</v>
       </c>
       <c r="D592" s="7" t="s">
         <v>32</v>
@@ -29304,7 +29329,7 @@
         <v>1</v>
       </c>
       <c r="H592" s="13" t="s">
-        <v>944</v>
+        <v>935</v>
       </c>
       <c r="M592" s="9" t="str" cm="1">
         <f t="array" ref="M592">PAGE_NAME(B592)</f>
@@ -29332,7 +29357,7 @@
         <v>327</v>
       </c>
       <c r="C593" s="8" t="s">
-        <v>1020</v>
+        <v>1011</v>
       </c>
       <c r="D593" s="7" t="s">
         <v>41</v>
@@ -29368,7 +29393,7 @@
         <v>327</v>
       </c>
       <c r="C594" s="8" t="s">
-        <v>1021</v>
+        <v>1012</v>
       </c>
       <c r="D594" s="7" t="s">
         <v>41</v>
@@ -29401,10 +29426,10 @@
         <v>702</v>
       </c>
       <c r="B595" s="23" t="s">
-        <v>1022</v>
+        <v>1013</v>
       </c>
       <c r="C595" s="8" t="s">
-        <v>1023</v>
+        <v>1014</v>
       </c>
       <c r="D595" s="7" t="s">
         <v>37</v>
@@ -29432,7 +29457,7 @@
         <v/>
       </c>
       <c r="U595" s="13" t="s">
-        <v>1024</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="596" spans="1:21" ht="51" x14ac:dyDescent="0.2">
@@ -29440,10 +29465,10 @@
         <v>703</v>
       </c>
       <c r="B596" s="23" t="s">
-        <v>1022</v>
+        <v>1013</v>
       </c>
       <c r="C596" s="8" t="s">
-        <v>1025</v>
+        <v>1016</v>
       </c>
       <c r="D596" s="7" t="s">
         <v>37</v>
@@ -29471,7 +29496,7 @@
         <v/>
       </c>
       <c r="U596" s="13" t="s">
-        <v>1026</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="597" spans="1:21" x14ac:dyDescent="0.2">
@@ -29535,7 +29560,7 @@
   <sheetData>
     <row r="1" spans="1:2" ht="409.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="69" t="s">
-        <v>1027</v>
+        <v>1018</v>
       </c>
       <c r="B1" s="70"/>
     </row>
@@ -29545,84 +29570,84 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="15" t="s">
-        <v>1028</v>
+        <v>1019</v>
       </c>
       <c r="B3" t="s">
-        <v>1059</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="15" t="s">
-        <v>1029</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="15" t="s">
-        <v>1030</v>
+        <v>1021</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>1031</v>
+        <v>1022</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="15" t="s">
-        <v>1032</v>
+        <v>1023</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>1033</v>
+        <v>1024</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="15" t="s">
-        <v>1034</v>
+        <v>1025</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>1035</v>
+        <v>1026</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="15" t="s">
-        <v>1036</v>
+        <v>1027</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>1037</v>
+        <v>1028</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="51" x14ac:dyDescent="0.2">
       <c r="A9" s="15" t="s">
-        <v>1038</v>
+        <v>1029</v>
       </c>
       <c r="B9" s="31" t="s">
-        <v>1039</v>
+        <v>1030</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" s="15" t="s">
-        <v>1040</v>
+        <v>1031</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="153" x14ac:dyDescent="0.2">
       <c r="A11" s="15" t="s">
-        <v>1041</v>
+        <v>1032</v>
       </c>
       <c r="B11" s="31" t="s">
-        <v>1042</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" s="15" t="s">
-        <v>1043</v>
+        <v>1034</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>1044</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" s="15" t="s">
-        <v>1045</v>
+        <v>1036</v>
       </c>
       <c r="B13" s="32" t="s">
-        <v>1046</v>
+        <v>1037</v>
       </c>
     </row>
   </sheetData>
@@ -29648,19 +29673,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="15" t="s">
-        <v>1030</v>
+        <v>1021</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>1047</v>
+        <v>1038</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>1048</v>
+        <v>1039</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>1049</v>
+        <v>1040</v>
       </c>
       <c r="E1" s="15" t="s">
-        <v>1050</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
@@ -29668,13 +29693,13 @@
         <v>0.1</v>
       </c>
       <c r="B2" t="s">
-        <v>1051</v>
+        <v>1042</v>
       </c>
       <c r="C2" s="44" t="s">
-        <v>1052</v>
+        <v>1043</v>
       </c>
       <c r="D2" t="s">
-        <v>1053</v>
+        <v>1044</v>
       </c>
       <c r="E2" s="45">
         <v>45618</v>
@@ -29695,13 +29720,13 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>1054</v>
+        <v>1045</v>
       </c>
       <c r="B1" t="s">
         <v>14</v>
       </c>
       <c r="C1" t="s">
-        <v>1055</v>
+        <v>1046</v>
       </c>
       <c r="D1" t="s">
         <v>16</v>
@@ -29718,7 +29743,7 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>1056</v>
+        <v>1047</v>
       </c>
       <c r="D2" t="s">
         <v>53</v>
@@ -29735,7 +29760,7 @@
         <v>0</v>
       </c>
       <c r="C3" t="s">
-        <v>1057</v>
+        <v>1048</v>
       </c>
       <c r="D3" t="s">
         <v>52</v>
@@ -29749,7 +29774,7 @@
         <v>41</v>
       </c>
       <c r="C4" t="s">
-        <v>1058</v>
+        <v>1049</v>
       </c>
       <c r="E4" t="s">
         <v>55</v>
@@ -29768,7 +29793,7 @@
         <v>75</v>
       </c>
       <c r="E6" t="s">
-        <v>877</v>
+        <v>870</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -29782,6 +29807,28 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="b5a44311-ed64-4a72-909f-c9dc6973bde2" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="eebd8b74-b9de-41b2-9247-c010c4973c2b">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Description xmlns="eebd8b74-b9de-41b2-9247-c010c4973c2b" xsi:nil="true"/>
+    <SortOrder xmlns="eebd8b74-b9de-41b2-9247-c010c4973c2b" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EC335ED7BB179244BF94A0DFE64544DC" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d3a0f66abe5d2a0564332877ab55d3f7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="eebd8b74-b9de-41b2-9247-c010c4973c2b" xmlns:ns3="b7009bbd-f938-489b-a530-f05273710fff" xmlns:ns4="b5a44311-ed64-4a72-909f-c9dc6973bde2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ec7ca2ee893ff8a0f61d4046c6461645" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="eebd8b74-b9de-41b2-9247-c010c4973c2b"/>
@@ -30035,29 +30082,33 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19B0E317-5E0E-4728-AB3F-40F2C2B957FB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="eebd8b74-b9de-41b2-9247-c010c4973c2b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="b7009bbd-f938-489b-a530-f05273710fff"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="b5a44311-ed64-4a72-909f-c9dc6973bde2"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="b5a44311-ed64-4a72-909f-c9dc6973bde2" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="eebd8b74-b9de-41b2-9247-c010c4973c2b">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Description xmlns="eebd8b74-b9de-41b2-9247-c010c4973c2b" xsi:nil="true"/>
-    <SortOrder xmlns="eebd8b74-b9de-41b2-9247-c010c4973c2b" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA84097F-5807-4DCF-92C6-48C9EE26CFB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C0B0A19-6928-4F0B-831A-5B9FDDD3F6CE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -30075,30 +30126,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA84097F-5807-4DCF-92C6-48C9EE26CFB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19B0E317-5E0E-4728-AB3F-40F2C2B957FB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="eebd8b74-b9de-41b2-9247-c010c4973c2b"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="b7009bbd-f938-489b-a530-f05273710fff"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="b5a44311-ed64-4a72-909f-c9dc6973bde2"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>